<commit_message>
Ethics and ML Results
</commit_message>
<xml_diff>
--- a/assets/data/Scores.xlsx
+++ b/assets/data/Scores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/23750492_stu_mmu_ac_uk/Documents/Documents/02. Evidence/05. Submission Feedback/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stuar\Documents\Personal\Studvart.github.io\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{AC7C8104-06E0-451F-91A0-1BFEDFC6BC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FD56E6F-3347-45AE-8DAF-F2161000619D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10D4CBA-DE9C-42DF-ACA3-9604D7D00C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="38670" windowHeight="21150" xr2:uid="{901B348F-9C94-4721-9324-85630299E8C4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{901B348F-9C94-4721-9324-85630299E8C4}"/>
   </bookViews>
   <sheets>
     <sheet name="Scores" sheetId="1" r:id="rId1"/>
@@ -207,7 +207,7 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -550,15 +550,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35B3BEE-B029-45ED-8870-AE1B43C3D377}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="67" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -575,7 +575,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>4</v>
       </c>
@@ -592,7 +592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>4</v>
       </c>
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>4</v>
       </c>
@@ -626,7 +626,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -643,7 +643,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -660,7 +660,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>4</v>
       </c>
@@ -677,7 +677,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -694,7 +694,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>4</v>
       </c>
@@ -711,7 +711,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>4</v>
       </c>
@@ -728,7 +728,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>5</v>
       </c>
@@ -745,7 +745,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>5</v>
       </c>
@@ -762,7 +762,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>5</v>
       </c>
@@ -779,7 +779,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>5</v>
       </c>
@@ -796,7 +796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -813,7 +813,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>5</v>
       </c>
@@ -826,9 +826,11 @@
       <c r="D16" s="6">
         <v>1</v>
       </c>
-      <c r="E16" s="6"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E16" s="6">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>6</v>
       </c>
@@ -841,9 +843,11 @@
       <c r="D17" s="7">
         <v>1</v>
       </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="7">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>6</v>
       </c>
@@ -854,7 +858,7 @@
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>6</v>
       </c>
@@ -865,7 +869,7 @@
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>6</v>
       </c>

</xml_diff>